<commit_message>
24_25_isik veri dosyasina Dil kolonu eklendi
</commit_message>
<xml_diff>
--- a/24_25_isik (1).xlsx
+++ b/24_25_isik (1).xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\selection_project2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\IDARI\OgrenciIsleriDB\OIDB Server\CİHAN TAZEÖZ\Uygulamalar\selection_project2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F55F85A5-9641-4705-AACB-C9DD326B06E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C1C750-788B-4F32-85DD-2245F70A53B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
     <sheet name="Sayfa2" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sayfa1!$A$1:$H$109</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sayfa1!$A$1:$I$109</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="634" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="240">
   <si>
     <t>Fakülte/Yüksekokul Adı</t>
   </si>
@@ -751,6 +751,15 @@
   </si>
   <si>
     <t>ULUSLARARASI TİCARET VE FİNANSMAN (İNGİLİZCE) (ÜCRETLİ)</t>
+  </si>
+  <si>
+    <t>Dil</t>
+  </si>
+  <si>
+    <t>ING</t>
+  </si>
+  <si>
+    <t>TR</t>
   </si>
 </sst>
 </file>
@@ -797,6 +806,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
       <charset val="162"/>
     </font>
     <font>
@@ -1207,21 +1217,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H109"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I109"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.109375" customWidth="1"/>
-    <col min="2" max="2" width="78.44140625" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="44.140625" customWidth="1"/>
+    <col min="2" max="2" width="78.42578125" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.21875" customWidth="1"/>
-    <col min="6" max="6" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1246,8 +1256,11 @@
       <c r="H1" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I1" s="2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1272,8 +1285,11 @@
       <c r="H2" s="8" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I2" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>46</v>
       </c>
@@ -1298,8 +1314,11 @@
       <c r="H3" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I3" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>46</v>
       </c>
@@ -1324,8 +1343,11 @@
       <c r="H4" s="8" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I4" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>46</v>
       </c>
@@ -1350,8 +1372,11 @@
       <c r="H5" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I5" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>46</v>
       </c>
@@ -1376,8 +1401,11 @@
       <c r="H6" s="8" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I6" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>19</v>
       </c>
@@ -1402,8 +1430,11 @@
       <c r="H7" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I7" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>19</v>
       </c>
@@ -1428,8 +1459,11 @@
       <c r="H8" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I8" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>19</v>
       </c>
@@ -1454,8 +1488,11 @@
       <c r="H9" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I9" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>46</v>
       </c>
@@ -1480,8 +1517,11 @@
       <c r="H10" s="8" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I10" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>46</v>
       </c>
@@ -1506,8 +1546,11 @@
       <c r="H11" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I11" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>46</v>
       </c>
@@ -1532,8 +1575,11 @@
       <c r="H12" s="8" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I12" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>46</v>
       </c>
@@ -1558,8 +1604,11 @@
       <c r="H13" s="8" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I13" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>46</v>
       </c>
@@ -1584,8 +1633,11 @@
       <c r="H14" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I14" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>46</v>
       </c>
@@ -1610,8 +1662,11 @@
       <c r="H15" s="8" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I15" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>19</v>
       </c>
@@ -1636,8 +1691,11 @@
       <c r="H16" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I16" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -1662,8 +1720,11 @@
       <c r="H17" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I17" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>46</v>
       </c>
@@ -1688,8 +1749,11 @@
       <c r="H18" s="8" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I18" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>46</v>
       </c>
@@ -1714,8 +1778,11 @@
       <c r="H19" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I19" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>46</v>
       </c>
@@ -1740,8 +1807,11 @@
       <c r="H20" s="8" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I20" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>19</v>
       </c>
@@ -1766,8 +1836,11 @@
       <c r="H21" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I21" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>19</v>
       </c>
@@ -1792,8 +1865,11 @@
       <c r="H22" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I22" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>19</v>
       </c>
@@ -1818,8 +1894,11 @@
       <c r="H23" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I23" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>19</v>
       </c>
@@ -1844,8 +1923,11 @@
       <c r="H24" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I24" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>19</v>
       </c>
@@ -1870,8 +1952,11 @@
       <c r="H25" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I25" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>33</v>
       </c>
@@ -1896,8 +1981,11 @@
       <c r="H26" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I26" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>33</v>
       </c>
@@ -1922,8 +2010,11 @@
       <c r="H27" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I27" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>33</v>
       </c>
@@ -1948,8 +2039,11 @@
       <c r="H28" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I28" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>33</v>
       </c>
@@ -1974,8 +2068,11 @@
       <c r="H29" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I29" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>33</v>
       </c>
@@ -2000,8 +2097,11 @@
       <c r="H30" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I30" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>33</v>
       </c>
@@ -2026,8 +2126,11 @@
       <c r="H31" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I31" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>46</v>
       </c>
@@ -2052,8 +2155,11 @@
       <c r="H32" s="8" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I32" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>46</v>
       </c>
@@ -2078,8 +2184,11 @@
       <c r="H33" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I33" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>46</v>
       </c>
@@ -2104,8 +2213,11 @@
       <c r="H34" s="8" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I34" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>33</v>
       </c>
@@ -2130,8 +2242,11 @@
       <c r="H35" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I35" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>33</v>
       </c>
@@ -2156,8 +2271,11 @@
       <c r="H36" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I36" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>33</v>
       </c>
@@ -2182,8 +2300,11 @@
       <c r="H37" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I37" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>33</v>
       </c>
@@ -2208,8 +2329,11 @@
       <c r="H38" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I38" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>33</v>
       </c>
@@ -2234,8 +2358,11 @@
       <c r="H39" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I39" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>33</v>
       </c>
@@ -2260,8 +2387,11 @@
       <c r="H40" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I40" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>6</v>
       </c>
@@ -2286,8 +2416,11 @@
       <c r="H41" s="8" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I41" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>6</v>
       </c>
@@ -2312,8 +2445,11 @@
       <c r="H42" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I42" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>46</v>
       </c>
@@ -2338,8 +2474,11 @@
       <c r="H43" s="8" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I43" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>46</v>
       </c>
@@ -2364,8 +2503,11 @@
       <c r="H44" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I44" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>46</v>
       </c>
@@ -2390,8 +2532,11 @@
       <c r="H45" s="8" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I45" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>19</v>
       </c>
@@ -2416,8 +2561,11 @@
       <c r="H46" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I46" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>19</v>
       </c>
@@ -2442,8 +2590,11 @@
       <c r="H47" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I47" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>6</v>
       </c>
@@ -2468,8 +2619,11 @@
       <c r="H48" s="8" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I48" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>6</v>
       </c>
@@ -2494,8 +2648,11 @@
       <c r="H49" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I49" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
         <v>19</v>
       </c>
@@ -2520,8 +2677,11 @@
       <c r="H50" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I50" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
         <v>19</v>
       </c>
@@ -2546,8 +2706,11 @@
       <c r="H51" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I51" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
         <v>19</v>
       </c>
@@ -2572,8 +2735,11 @@
       <c r="H52" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I52" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
         <v>19</v>
       </c>
@@ -2598,8 +2764,11 @@
       <c r="H53" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I53" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
         <v>33</v>
       </c>
@@ -2618,8 +2787,11 @@
       <c r="H54" s="11" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I54" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>33</v>
       </c>
@@ -2638,8 +2810,11 @@
       <c r="H55" s="11" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I55" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
         <v>46</v>
       </c>
@@ -2664,8 +2839,11 @@
       <c r="H56" s="8" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I56" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
         <v>46</v>
       </c>
@@ -2690,8 +2868,11 @@
       <c r="H57" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I57" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
         <v>46</v>
       </c>
@@ -2716,8 +2897,11 @@
       <c r="H58" s="8" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I58" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
         <v>6</v>
       </c>
@@ -2742,8 +2926,11 @@
       <c r="H59" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I59" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
         <v>6</v>
       </c>
@@ -2768,8 +2955,11 @@
       <c r="H60" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I60" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
         <v>6</v>
       </c>
@@ -2794,8 +2984,11 @@
       <c r="H61" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I61" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
         <v>6</v>
       </c>
@@ -2820,8 +3013,11 @@
       <c r="H62" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I62" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
         <v>6</v>
       </c>
@@ -2846,8 +3042,11 @@
       <c r="H63" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I63" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
         <v>6</v>
       </c>
@@ -2872,8 +3071,11 @@
       <c r="H64" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I64" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
         <v>33</v>
       </c>
@@ -2898,8 +3100,11 @@
       <c r="H65" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I65" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
         <v>33</v>
       </c>
@@ -2924,8 +3129,11 @@
       <c r="H66" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I66" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
         <v>33</v>
       </c>
@@ -2950,8 +3158,11 @@
       <c r="H67" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I67" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
         <v>46</v>
       </c>
@@ -2976,8 +3187,11 @@
       <c r="H68" s="8" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I68" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>46</v>
       </c>
@@ -3002,8 +3216,11 @@
       <c r="H69" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I69" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
         <v>46</v>
       </c>
@@ -3028,8 +3245,11 @@
       <c r="H70" s="8" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I70" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
         <v>46</v>
       </c>
@@ -3054,8 +3274,11 @@
       <c r="H71" s="8" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I71" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
         <v>46</v>
       </c>
@@ -3080,8 +3303,11 @@
       <c r="H72" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I72" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
         <v>6</v>
       </c>
@@ -3106,8 +3332,11 @@
       <c r="H73" s="8" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I73" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
         <v>6</v>
       </c>
@@ -3132,8 +3361,11 @@
       <c r="H74" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I74" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
         <v>6</v>
       </c>
@@ -3152,8 +3384,11 @@
       <c r="H75" s="11" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I75" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
         <v>33</v>
       </c>
@@ -3172,8 +3407,11 @@
       <c r="H76" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I76" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
         <v>19</v>
       </c>
@@ -3198,8 +3436,11 @@
       <c r="H77" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I77" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
         <v>19</v>
       </c>
@@ -3224,8 +3465,11 @@
       <c r="H78" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I78" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
         <v>19</v>
       </c>
@@ -3250,8 +3494,11 @@
       <c r="H79" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I79" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
         <v>6</v>
       </c>
@@ -3276,8 +3523,11 @@
       <c r="H80" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I80" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
         <v>6</v>
       </c>
@@ -3302,8 +3552,11 @@
       <c r="H81" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I81" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
         <v>6</v>
       </c>
@@ -3328,8 +3581,11 @@
       <c r="H82" s="8" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I82" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
         <v>6</v>
       </c>
@@ -3354,8 +3610,11 @@
       <c r="H83" s="8" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I83" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
         <v>6</v>
       </c>
@@ -3380,8 +3639,11 @@
       <c r="H84" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I84" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
         <v>6</v>
       </c>
@@ -3406,8 +3668,11 @@
       <c r="H85" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I85" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
         <v>6</v>
       </c>
@@ -3426,8 +3691,11 @@
       <c r="H86" s="10" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I86" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
         <v>6</v>
       </c>
@@ -3444,8 +3712,11 @@
       <c r="H87" s="10" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I87" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
         <v>6</v>
       </c>
@@ -3462,8 +3733,11 @@
       <c r="H88" s="10" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I88" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
         <v>6</v>
       </c>
@@ -3480,8 +3754,11 @@
       <c r="H89" s="10" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I89" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
         <v>6</v>
       </c>
@@ -3498,8 +3775,11 @@
       <c r="H90" s="10" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I90" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
         <v>6</v>
       </c>
@@ -3518,8 +3798,11 @@
       <c r="H91" s="11" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I91" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
         <v>6</v>
       </c>
@@ -3538,8 +3821,11 @@
       <c r="H92" s="10" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I92" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
         <v>6</v>
       </c>
@@ -3558,8 +3844,11 @@
       <c r="H93" s="10" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I93" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
         <v>6</v>
       </c>
@@ -3584,8 +3873,11 @@
       <c r="H94" s="10" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I94" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
         <v>6</v>
       </c>
@@ -3610,8 +3902,11 @@
       <c r="H95" s="10" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I95" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
         <v>19</v>
       </c>
@@ -3628,8 +3923,11 @@
       <c r="H96" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I96" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
         <v>19</v>
       </c>
@@ -3646,8 +3944,11 @@
       <c r="H97" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I97" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
         <v>19</v>
       </c>
@@ -3664,8 +3965,11 @@
       <c r="H98" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I98" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
         <v>19</v>
       </c>
@@ -3682,8 +3986,11 @@
       <c r="H99" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I99" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
         <v>19</v>
       </c>
@@ -3700,8 +4007,11 @@
       <c r="H100" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I100" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
         <v>33</v>
       </c>
@@ -3726,8 +4036,11 @@
       <c r="H101" s="10" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I101" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" s="5" t="s">
         <v>33</v>
       </c>
@@ -3752,8 +4065,11 @@
       <c r="H102" s="10" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I102" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" s="5" t="s">
         <v>33</v>
       </c>
@@ -3772,8 +4088,11 @@
       <c r="H103" s="10" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I103" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" s="5" t="s">
         <v>6</v>
       </c>
@@ -3792,8 +4111,11 @@
       <c r="H104" s="10" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I104" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" s="5" t="s">
         <v>46</v>
       </c>
@@ -3810,8 +4132,11 @@
       <c r="H105" s="10" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I105" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" s="5" t="s">
         <v>46</v>
       </c>
@@ -3828,8 +4153,11 @@
       <c r="H106" s="10" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I106" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" s="5" t="s">
         <v>46</v>
       </c>
@@ -3846,8 +4174,11 @@
       <c r="H107" s="10" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I107" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" s="5" t="s">
         <v>46</v>
       </c>
@@ -3864,8 +4195,11 @@
       <c r="H108" s="10" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="I108" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" s="5" t="s">
         <v>46</v>
       </c>
@@ -3882,20 +4216,11 @@
       <c r="H109" s="10" t="s">
         <v>125</v>
       </c>
+      <c r="I109" s="5" t="s">
+        <v>239</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H109" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="DIŞ TİCARET (%50 İNDİRİMLİ)"/>
-        <filter val="DIŞ TİCARET (BURSLU)"/>
-        <filter val="DIŞ TİCARET (ÜCRETLİ)"/>
-        <filter val="ULUSLARARASI TİCARET (İNGİLİZCE) (ÜCRETLİ)"/>
-        <filter val="ULUSLARARASI TİCARET VE FİNANSMAN (İNGİLİZCE) (%50 İNDİRİMLİ)"/>
-        <filter val="ULUSLARARASI TİCARET VE FİNANSMAN (İNGİLİZCE) (BURSLU)"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
@@ -3907,13 +4232,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B2B85CB-6E4F-48DB-B608-11A2F2B856AB}">
   <dimension ref="A1:B94"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="44.44140625" customWidth="1"/>
-    <col min="2" max="2" width="20.88671875" customWidth="1"/>
+    <col min="1" max="1" width="44.42578125" customWidth="1"/>
+    <col min="2" max="2" width="20.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>13</v>
       </c>
@@ -3921,7 +4246,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>10</v>
       </c>
@@ -3929,7 +4254,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>12</v>
       </c>
@@ -3937,7 +4262,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>11</v>
       </c>
@@ -3945,7 +4270,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>18</v>
       </c>
@@ -3953,7 +4278,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>15</v>
       </c>
@@ -3961,7 +4286,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>17</v>
       </c>
@@ -3969,7 +4294,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>16</v>
       </c>
@@ -3977,7 +4302,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>83</v>
       </c>
@@ -3985,7 +4310,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>7</v>
       </c>
@@ -3993,7 +4318,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>86</v>
       </c>
@@ -4001,7 +4326,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>9</v>
       </c>
@@ -4009,7 +4334,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>87</v>
       </c>
@@ -4017,7 +4342,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>114</v>
       </c>
@@ -4025,7 +4350,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>106</v>
       </c>
@@ -4033,7 +4358,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>14</v>
       </c>
@@ -4041,7 +4366,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>116</v>
       </c>
@@ -4049,7 +4374,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>117</v>
       </c>
@@ -4057,7 +4382,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>88</v>
       </c>
@@ -4065,7 +4390,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>115</v>
       </c>
@@ -4073,7 +4398,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>22</v>
       </c>
@@ -4081,7 +4406,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>20</v>
       </c>
@@ -4089,7 +4414,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>118</v>
       </c>
@@ -4097,7 +4422,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>23</v>
       </c>
@@ -4105,7 +4430,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>119</v>
       </c>
@@ -4113,7 +4438,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>24</v>
       </c>
@@ -4121,7 +4446,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>26</v>
       </c>
@@ -4129,7 +4454,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>25</v>
       </c>
@@ -4137,7 +4462,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>89</v>
       </c>
@@ -4145,7 +4470,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>28</v>
       </c>
@@ -4153,7 +4478,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>90</v>
       </c>
@@ -4161,7 +4486,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>29</v>
       </c>
@@ -4169,7 +4494,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
         <v>107</v>
       </c>
@@ -4177,7 +4502,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>30</v>
       </c>
@@ -4185,7 +4510,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="9" t="s">
         <v>32</v>
       </c>
@@ -4193,7 +4518,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
         <v>31</v>
       </c>
@@ -4201,7 +4526,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
         <v>35</v>
       </c>
@@ -4209,7 +4534,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
         <v>34</v>
       </c>
@@ -4217,7 +4542,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="9" t="s">
         <v>41</v>
       </c>
@@ -4225,7 +4550,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="9" t="s">
         <v>40</v>
       </c>
@@ -4233,7 +4558,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="9" t="s">
         <v>91</v>
       </c>
@@ -4241,7 +4566,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="9" t="s">
         <v>108</v>
       </c>
@@ -4249,7 +4574,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="9" t="s">
         <v>92</v>
       </c>
@@ -4257,7 +4582,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="9" t="s">
         <v>43</v>
       </c>
@@ -4265,7 +4590,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="9" t="s">
         <v>38</v>
       </c>
@@ -4273,7 +4598,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="9" t="s">
         <v>36</v>
       </c>
@@ -4281,7 +4606,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="9" t="s">
         <v>42</v>
       </c>
@@ -4289,7 +4614,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="9" t="s">
         <v>39</v>
       </c>
@@ -4297,7 +4622,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="9" t="s">
         <v>45</v>
       </c>
@@ -4305,7 +4630,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" s="9" t="s">
         <v>44</v>
       </c>
@@ -4313,7 +4638,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" s="9" t="s">
         <v>93</v>
       </c>
@@ -4321,7 +4646,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" s="9" t="s">
         <v>47</v>
       </c>
@@ -4329,7 +4654,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" s="9" t="s">
         <v>100</v>
       </c>
@@ -4337,7 +4662,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" s="9" t="s">
         <v>49</v>
       </c>
@@ -4345,7 +4670,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" s="9" t="s">
         <v>51</v>
       </c>
@@ -4353,7 +4678,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" s="9" t="s">
         <v>50</v>
       </c>
@@ -4361,7 +4686,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" s="9" t="s">
         <v>101</v>
       </c>
@@ -4369,7 +4694,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" s="9" t="s">
         <v>109</v>
       </c>
@@ -4377,7 +4702,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" s="9" t="s">
         <v>55</v>
       </c>
@@ -4385,7 +4710,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" s="9" t="s">
         <v>52</v>
       </c>
@@ -4393,7 +4718,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" s="9" t="s">
         <v>54</v>
       </c>
@@ -4401,7 +4726,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" s="9" t="s">
         <v>53</v>
       </c>
@@ -4409,7 +4734,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" s="9" t="s">
         <v>59</v>
       </c>
@@ -4417,7 +4742,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" s="9" t="s">
         <v>58</v>
       </c>
@@ -4425,7 +4750,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="9" t="s">
         <v>102</v>
       </c>
@@ -4433,7 +4758,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" s="9" t="s">
         <v>110</v>
       </c>
@@ -4441,7 +4766,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" s="9" t="s">
         <v>63</v>
       </c>
@@ -4449,7 +4774,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" s="9" t="s">
         <v>60</v>
       </c>
@@ -4457,7 +4782,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" s="9" t="s">
         <v>62</v>
       </c>
@@ -4465,7 +4790,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" s="9" t="s">
         <v>61</v>
       </c>
@@ -4473,7 +4798,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" s="9" t="s">
         <v>67</v>
       </c>
@@ -4481,7 +4806,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" s="9" t="s">
         <v>64</v>
       </c>
@@ -4489,7 +4814,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" s="9" t="s">
         <v>66</v>
       </c>
@@ -4497,7 +4822,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" s="9" t="s">
         <v>65</v>
       </c>
@@ -4505,7 +4830,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" s="9" t="s">
         <v>71</v>
       </c>
@@ -4513,7 +4838,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" s="9" t="s">
         <v>68</v>
       </c>
@@ -4521,7 +4846,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" s="9" t="s">
         <v>70</v>
       </c>
@@ -4529,7 +4854,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" s="9" t="s">
         <v>69</v>
       </c>
@@ -4537,7 +4862,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" s="9" t="s">
         <v>75</v>
       </c>
@@ -4545,7 +4870,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" s="9" t="s">
         <v>72</v>
       </c>
@@ -4553,7 +4878,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="9" t="s">
         <v>74</v>
       </c>
@@ -4561,7 +4886,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A82" s="9" t="s">
         <v>73</v>
       </c>
@@ -4569,7 +4894,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" s="9" t="s">
         <v>98</v>
       </c>
@@ -4577,7 +4902,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" s="9" t="s">
         <v>76</v>
       </c>
@@ -4585,7 +4910,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" s="9" t="s">
         <v>103</v>
       </c>
@@ -4593,7 +4918,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" s="9" t="s">
         <v>77</v>
       </c>
@@ -4601,7 +4926,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" s="9" t="s">
         <v>57</v>
       </c>
@@ -4609,7 +4934,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" s="9" t="s">
         <v>56</v>
       </c>
@@ -4617,7 +4942,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" s="9" t="s">
         <v>104</v>
       </c>
@@ -4625,7 +4950,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" s="9" t="s">
         <v>111</v>
       </c>
@@ -4633,7 +4958,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" s="9" t="s">
         <v>99</v>
       </c>
@@ -4641,7 +4966,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" s="9" t="s">
         <v>112</v>
       </c>
@@ -4649,7 +4974,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" s="9" t="s">
         <v>105</v>
       </c>
@@ -4657,7 +4982,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" s="9" t="s">
         <v>113</v>
       </c>
@@ -4671,6 +4996,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="419a74c1-09a2-4307-93c4-563b7c0144a0" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Belge" ma:contentTypeID="0x010100F4C584498243654AA32BFFB3F8F1F718" ma:contentTypeVersion="10" ma:contentTypeDescription="Yeni belge oluşturun." ma:contentTypeScope="" ma:versionID="deaa675999c720fb8c611846574709b5">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="419a74c1-09a2-4307-93c4-563b7c0144a0" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="dcc3ec335f4ea9ff4a71c58e3178d539" ns3:_="">
     <xsd:import namespace="419a74c1-09a2-4307-93c4-563b7c0144a0"/>
@@ -4852,24 +5194,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17F7ABFD-B3B5-4850-953C-399810998E16}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="419a74c1-09a2-4307-93c4-563b7c0144a0"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="419a74c1-09a2-4307-93c4-563b7c0144a0" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAAE7014-3F90-4318-B766-25DF7CB6C87E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A436612-0B66-40B4-A512-333F88791E2E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4885,28 +5234,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CAAE7014-3F90-4318-B766-25DF7CB6C87E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17F7ABFD-B3B5-4850-953C-399810998E16}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="419a74c1-09a2-4307-93c4-563b7c0144a0"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
PDF indirme eklendi, ucret formatlamasi ve kvkk metni guncellendi
</commit_message>
<xml_diff>
--- a/24_25_isik (1).xlsx
+++ b/24_25_isik (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\IDARI\OgrenciIsleriDB\OIDB Server\CİHAN TAZEÖZ\Uygulamalar\selection_project2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1C1C750-788B-4F32-85DD-2245F70A53B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E7B1D8-65C6-4FE7-8B9B-9600A70F6CEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="240">
   <si>
     <t>Fakülte/Yüksekokul Adı</t>
   </si>
@@ -2778,12 +2778,18 @@
       <c r="C54" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D54" s="1" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E54" s="10"/>
-      <c r="F54" s="10"/>
-      <c r="G54" s="10"/>
+      <c r="D54" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G54" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="H54" s="11" t="s">
         <v>121</v>
       </c>
@@ -2801,12 +2807,18 @@
       <c r="C55" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D55" s="1" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E55" s="10"/>
-      <c r="F55" s="10"/>
-      <c r="G55" s="10"/>
+      <c r="D55" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G55" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="H55" s="11" t="s">
         <v>122</v>
       </c>
@@ -3398,12 +3410,18 @@
       <c r="C76" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D76" s="1" t="e">
-        <v>#N/A</v>
-      </c>
-      <c r="E76" s="10"/>
-      <c r="F76" s="10"/>
-      <c r="G76" s="10"/>
+      <c r="D76" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E76" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F76" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G76" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="H76" s="10" t="s">
         <v>120</v>
       </c>
@@ -4082,9 +4100,15 @@
       <c r="D103" s="1">
         <v>0</v>
       </c>
-      <c r="E103" s="10"/>
-      <c r="F103" s="10"/>
-      <c r="G103" s="10"/>
+      <c r="E103" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="F103" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G103" s="10" t="s">
+        <v>79</v>
+      </c>
       <c r="H103" s="10" t="s">
         <v>120</v>
       </c>

</xml_diff>